<commit_message>
Update NY gaming data - Fri Oct 30 17:21:04 UTC 2026
</commit_message>
<xml_diff>
--- a/NY_State_Reports_2026-10-30/Bally_Bet_Weekly_Report.xlsx
+++ b/NY_State_Reports_2026-10-30/Bally_Bet_Weekly_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\MOBILE SPORTS WAGERING\11_Weekly Web Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D512856C-85EA-4678-B919-805F00A19B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1375C35-16B6-4802-88C4-2E1DAC48CE2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EDA5EF8F-B63B-4D9E-966F-AB4A019BBE74}"/>
   </bookViews>
@@ -2868,7 +2868,12 @@
         <v>46320</v>
       </c>
       <c r="B43" s="20"/>
-      <c r="F43" s="23"/>
+      <c r="C43" s="21">
+        <v>3547164.3500000006</v>
+      </c>
+      <c r="F43" s="23">
+        <v>422608.17</v>
+      </c>
       <c r="G43"/>
       <c r="H43"/>
       <c r="I43"/>
@@ -3368,11 +3373,11 @@
       </c>
       <c r="C67" s="24">
         <f>SUM(C13:C66)</f>
-        <v>90656906.070000008</v>
+        <v>94204070.420000002</v>
       </c>
       <c r="F67" s="24">
         <f>SUM(F13:F66)</f>
-        <v>8225592.6100000003</v>
+        <v>8648200.7800000012</v>
       </c>
       <c r="G67"/>
       <c r="H67"/>

</xml_diff>